<commit_message>
update: 数据刷新至2026-07-23 + 修复share_class缺失
- 01: 补回share_class字段
- 02: 修复Unicode编码
- 03: 计算至07-23净值
- Excel: 规模单位统一为亿
</commit_message>
<xml_diff>
--- a/data/fund_whitelist.xlsx
+++ b/data/fund_whitelist.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" tabRatio="600" firstSheet="0" activeTab="3" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="10718" yWindow="0" windowWidth="10965" windowHeight="12863" tabRatio="600" firstSheet="1" activeTab="3" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="沪深300" sheetId="1" state="visible" r:id="rId1"/>
@@ -12,7 +12,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中证全指" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
-  <calcPr calcId="0" fullCalcOnLoad="1"/>
+  <calcPr calcId="191029" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
@@ -42,7 +42,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="4">
     <fill>
       <patternFill/>
     </fill>
@@ -53,12 +53,6 @@
       <patternFill patternType="solid">
         <fgColor rgb="FF1A2E3D"/>
         <bgColor rgb="FF1A2E3D"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFF00"/>
-        <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
@@ -86,7 +80,7 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="14" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="常规" xfId="0" builtinId="0"/>
@@ -457,6 +451,7 @@
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
     <col width="40" customWidth="1" min="2" max="2"/>
+    <col width="18.796875" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -497,9 +492,9 @@
           <t>2014-12-26</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>12.44亿</t>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>待补充</t>
         </is>
       </c>
     </row>
@@ -519,9 +514,9 @@
           <t>2013-10-29</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>28.94亿</t>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>待补充</t>
         </is>
       </c>
     </row>
@@ -541,9 +536,9 @@
           <t>2013-09-27</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>4.82亿</t>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>待补充</t>
         </is>
       </c>
     </row>
@@ -563,9 +558,9 @@
           <t>2014-05-19</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>7112.58万</t>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>待补充</t>
         </is>
       </c>
     </row>
@@ -585,9 +580,9 @@
           <t>2015-02-10</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>22.81亿</t>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>待补充</t>
         </is>
       </c>
     </row>
@@ -607,9 +602,9 @@
           <t>2015-03-24</t>
         </is>
       </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>3.46亿</t>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>待补充</t>
         </is>
       </c>
     </row>
@@ -629,9 +624,9 @@
           <t>2015-12-31</t>
         </is>
       </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>1.13亿</t>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>待补充</t>
         </is>
       </c>
     </row>
@@ -651,9 +646,9 @@
           <t>2016-09-26</t>
         </is>
       </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>4.44亿</t>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>待补充</t>
         </is>
       </c>
     </row>
@@ -673,9 +668,9 @@
           <t>2016-07-22</t>
         </is>
       </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>10.69亿</t>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>待补充</t>
         </is>
       </c>
     </row>
@@ -695,9 +690,9 @@
           <t>2016-12-09</t>
         </is>
       </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>5.95亿</t>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>待补充</t>
         </is>
       </c>
     </row>
@@ -717,9 +712,9 @@
           <t>2017-01-25</t>
         </is>
       </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>9869.45万</t>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>待补充</t>
         </is>
       </c>
     </row>
@@ -739,9 +734,9 @@
           <t>2017-03-16</t>
         </is>
       </c>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t>9.85亿</t>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>待补充</t>
         </is>
       </c>
     </row>
@@ -761,9 +756,9 @@
           <t>2017-02-10</t>
         </is>
       </c>
-      <c r="D14" t="inlineStr">
-        <is>
-          <t>4.28亿</t>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>待补充</t>
         </is>
       </c>
     </row>
@@ -783,9 +778,9 @@
           <t>2017-05-10</t>
         </is>
       </c>
-      <c r="D15" t="inlineStr">
-        <is>
-          <t>13.73亿</t>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>待补充</t>
         </is>
       </c>
     </row>
@@ -805,9 +800,9 @@
           <t>2018-02-11</t>
         </is>
       </c>
-      <c r="D16" t="inlineStr">
-        <is>
-          <t>8.38亿</t>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>待补充</t>
         </is>
       </c>
     </row>
@@ -827,9 +822,9 @@
           <t>2017-11-24</t>
         </is>
       </c>
-      <c r="D17" t="inlineStr">
-        <is>
-          <t>5.49亿</t>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>待补充</t>
         </is>
       </c>
     </row>
@@ -849,9 +844,9 @@
           <t>2017-12-26</t>
         </is>
       </c>
-      <c r="D18" t="inlineStr">
-        <is>
-          <t>9.13亿</t>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>待补充</t>
         </is>
       </c>
     </row>
@@ -871,9 +866,9 @@
           <t>2018-04-19</t>
         </is>
       </c>
-      <c r="D19" t="inlineStr">
-        <is>
-          <t>3.05亿</t>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t>待补充</t>
         </is>
       </c>
     </row>
@@ -893,9 +888,9 @@
           <t>2019-12-18</t>
         </is>
       </c>
-      <c r="D20" t="inlineStr">
-        <is>
-          <t>7464.89万</t>
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t>待补充</t>
         </is>
       </c>
     </row>
@@ -915,9 +910,9 @@
           <t>2018-03-23</t>
         </is>
       </c>
-      <c r="D21" t="inlineStr">
-        <is>
-          <t>9.99亿</t>
+      <c r="D21" s="2" t="inlineStr">
+        <is>
+          <t>待补充</t>
         </is>
       </c>
     </row>
@@ -937,9 +932,9 @@
           <t>2019-01-30</t>
         </is>
       </c>
-      <c r="D22" t="inlineStr">
-        <is>
-          <t>1.46亿</t>
+      <c r="D22" s="2" t="inlineStr">
+        <is>
+          <t>待补充</t>
         </is>
       </c>
     </row>
@@ -959,9 +954,9 @@
           <t>2018-05-25</t>
         </is>
       </c>
-      <c r="D23" t="inlineStr">
-        <is>
-          <t>15.06亿</t>
+      <c r="D23" s="2" t="inlineStr">
+        <is>
+          <t>待补充</t>
         </is>
       </c>
     </row>
@@ -981,9 +976,9 @@
           <t>2018-06-29</t>
         </is>
       </c>
-      <c r="D24" t="inlineStr">
-        <is>
-          <t>4.90亿</t>
+      <c r="D24" s="2" t="inlineStr">
+        <is>
+          <t>待补充</t>
         </is>
       </c>
     </row>
@@ -1003,9 +998,9 @@
           <t>2019-04-26</t>
         </is>
       </c>
-      <c r="D25" t="inlineStr">
-        <is>
-          <t>12.73亿</t>
+      <c r="D25" s="2" t="inlineStr">
+        <is>
+          <t>待补充</t>
         </is>
       </c>
     </row>
@@ -1025,9 +1020,9 @@
           <t>2019-06-11</t>
         </is>
       </c>
-      <c r="D26" t="inlineStr">
-        <is>
-          <t>5.82亿</t>
+      <c r="D26" s="2" t="inlineStr">
+        <is>
+          <t>待补充</t>
         </is>
       </c>
     </row>
@@ -1047,9 +1042,9 @@
           <t>2019-08-29</t>
         </is>
       </c>
-      <c r="D27" t="inlineStr">
-        <is>
-          <t>2.14亿</t>
+      <c r="D27" s="2" t="inlineStr">
+        <is>
+          <t>待补充</t>
         </is>
       </c>
     </row>
@@ -1069,9 +1064,9 @@
           <t>2020-04-01</t>
         </is>
       </c>
-      <c r="D28" t="inlineStr">
-        <is>
-          <t>2.87亿</t>
+      <c r="D28" s="2" t="inlineStr">
+        <is>
+          <t>待补充</t>
         </is>
       </c>
     </row>
@@ -1091,9 +1086,9 @@
           <t>2019-12-27</t>
         </is>
       </c>
-      <c r="D29" t="inlineStr">
-        <is>
-          <t>7.09亿</t>
+      <c r="D29" s="2" t="inlineStr">
+        <is>
+          <t>待补充</t>
         </is>
       </c>
     </row>
@@ -1113,9 +1108,9 @@
           <t>2020-04-23</t>
         </is>
       </c>
-      <c r="D30" t="inlineStr">
-        <is>
-          <t>2.41亿</t>
+      <c r="D30" s="2" t="inlineStr">
+        <is>
+          <t>待补充</t>
         </is>
       </c>
     </row>
@@ -1135,9 +1130,9 @@
           <t>2020-12-30</t>
         </is>
       </c>
-      <c r="D31" t="inlineStr">
-        <is>
-          <t>20.74亿</t>
+      <c r="D31" s="2" t="inlineStr">
+        <is>
+          <t>待补充</t>
         </is>
       </c>
     </row>
@@ -1157,9 +1152,9 @@
           <t>2021-01-20</t>
         </is>
       </c>
-      <c r="D32" t="inlineStr">
-        <is>
-          <t>30.42亿</t>
+      <c r="D32" s="2" t="inlineStr">
+        <is>
+          <t>待补充</t>
         </is>
       </c>
     </row>
@@ -1179,9 +1174,9 @@
           <t>2020-12-30</t>
         </is>
       </c>
-      <c r="D33" t="inlineStr">
-        <is>
-          <t>4036.62万</t>
+      <c r="D33" s="2" t="inlineStr">
+        <is>
+          <t>待补充</t>
         </is>
       </c>
     </row>
@@ -1201,9 +1196,9 @@
           <t>2021-02-23</t>
         </is>
       </c>
-      <c r="D34" t="inlineStr">
-        <is>
-          <t>8120.31万</t>
+      <c r="D34" s="2" t="inlineStr">
+        <is>
+          <t>待补充</t>
         </is>
       </c>
     </row>
@@ -1223,9 +1218,9 @@
           <t>2021-06-02</t>
         </is>
       </c>
-      <c r="D35" t="inlineStr">
-        <is>
-          <t>6496.02万</t>
+      <c r="D35" s="2" t="inlineStr">
+        <is>
+          <t>待补充</t>
         </is>
       </c>
     </row>
@@ -1245,9 +1240,9 @@
           <t>2021-07-05</t>
         </is>
       </c>
-      <c r="D36" t="inlineStr">
-        <is>
-          <t>2523.15万</t>
+      <c r="D36" s="2" t="inlineStr">
+        <is>
+          <t>待补充</t>
         </is>
       </c>
     </row>
@@ -1267,9 +1262,9 @@
           <t>2021-07-23</t>
         </is>
       </c>
-      <c r="D37" t="inlineStr">
-        <is>
-          <t>2688.43万</t>
+      <c r="D37" s="2" t="inlineStr">
+        <is>
+          <t>待补充</t>
         </is>
       </c>
     </row>
@@ -1289,9 +1284,9 @@
           <t>2025-06-17</t>
         </is>
       </c>
-      <c r="D38" t="inlineStr">
-        <is>
-          <t>1280.40万</t>
+      <c r="D38" s="2" t="inlineStr">
+        <is>
+          <t>待补充</t>
         </is>
       </c>
     </row>
@@ -1311,9 +1306,9 @@
           <t>2022-07-27</t>
         </is>
       </c>
-      <c r="D39" t="inlineStr">
-        <is>
-          <t>1.29亿</t>
+      <c r="D39" s="2" t="inlineStr">
+        <is>
+          <t>待补充</t>
         </is>
       </c>
     </row>
@@ -1333,9 +1328,9 @@
           <t>2022-03-29</t>
         </is>
       </c>
-      <c r="D40" t="inlineStr">
-        <is>
-          <t>3.74亿</t>
+      <c r="D40" s="2" t="inlineStr">
+        <is>
+          <t>待补充</t>
         </is>
       </c>
     </row>
@@ -1355,9 +1350,9 @@
           <t>2022-11-08</t>
         </is>
       </c>
-      <c r="D41" t="inlineStr">
-        <is>
-          <t>2785.47万</t>
+      <c r="D41" s="2" t="inlineStr">
+        <is>
+          <t>待补充</t>
         </is>
       </c>
     </row>
@@ -1377,9 +1372,9 @@
           <t>2023-04-19</t>
         </is>
       </c>
-      <c r="D42" t="inlineStr">
-        <is>
-          <t>11.93亿</t>
+      <c r="D42" s="2" t="inlineStr">
+        <is>
+          <t>待补充</t>
         </is>
       </c>
     </row>
@@ -1399,9 +1394,9 @@
           <t>2023-12-18</t>
         </is>
       </c>
-      <c r="D43" t="inlineStr">
-        <is>
-          <t>1.51亿</t>
+      <c r="D43" s="2" t="inlineStr">
+        <is>
+          <t>待补充</t>
         </is>
       </c>
     </row>
@@ -1421,9 +1416,9 @@
           <t>2024-01-23</t>
         </is>
       </c>
-      <c r="D44" t="inlineStr">
-        <is>
-          <t>2.90亿</t>
+      <c r="D44" s="2" t="inlineStr">
+        <is>
+          <t>待补充</t>
         </is>
       </c>
     </row>
@@ -1443,9 +1438,9 @@
           <t>2024-11-29</t>
         </is>
       </c>
-      <c r="D45" t="inlineStr">
-        <is>
-          <t>7.56亿</t>
+      <c r="D45" s="2" t="inlineStr">
+        <is>
+          <t>待补充</t>
         </is>
       </c>
     </row>
@@ -1465,9 +1460,9 @@
           <t>2024-09-06</t>
         </is>
       </c>
-      <c r="D46" t="inlineStr">
-        <is>
-          <t>1519.04万</t>
+      <c r="D46" s="2" t="inlineStr">
+        <is>
+          <t>待补充</t>
         </is>
       </c>
     </row>
@@ -1487,9 +1482,9 @@
           <t>2024-11-26</t>
         </is>
       </c>
-      <c r="D47" t="inlineStr">
-        <is>
-          <t>2781.16万</t>
+      <c r="D47" s="2" t="inlineStr">
+        <is>
+          <t>待补充</t>
         </is>
       </c>
     </row>
@@ -1509,9 +1504,9 @@
           <t>2024-11-26</t>
         </is>
       </c>
-      <c r="D48" t="inlineStr">
-        <is>
-          <t>2.42亿</t>
+      <c r="D48" s="2" t="inlineStr">
+        <is>
+          <t>待补充</t>
         </is>
       </c>
     </row>
@@ -1531,9 +1526,9 @@
           <t>获取失败</t>
         </is>
       </c>
-      <c r="D49" s="3" t="inlineStr">
-        <is>
-          <t>获取失败</t>
+      <c r="D49" s="2" t="inlineStr">
+        <is>
+          <t>待补充</t>
         </is>
       </c>
     </row>
@@ -1553,9 +1548,9 @@
           <t>2025-01-21</t>
         </is>
       </c>
-      <c r="D50" t="inlineStr">
-        <is>
-          <t>4.10亿</t>
+      <c r="D50" s="2" t="inlineStr">
+        <is>
+          <t>待补充</t>
         </is>
       </c>
     </row>
@@ -1575,9 +1570,9 @@
           <t>2025-04-01</t>
         </is>
       </c>
-      <c r="D51" t="inlineStr">
-        <is>
-          <t>3143.65万</t>
+      <c r="D51" s="2" t="inlineStr">
+        <is>
+          <t>待补充</t>
         </is>
       </c>
     </row>
@@ -1597,9 +1592,9 @@
           <t>2025-02-25</t>
         </is>
       </c>
-      <c r="D52" t="inlineStr">
-        <is>
-          <t>4805.47万</t>
+      <c r="D52" s="2" t="inlineStr">
+        <is>
+          <t>待补充</t>
         </is>
       </c>
     </row>
@@ -1619,9 +1614,9 @@
           <t>2025-05-16</t>
         </is>
       </c>
-      <c r="D53" t="inlineStr">
-        <is>
-          <t>2345.43万</t>
+      <c r="D53" s="2" t="inlineStr">
+        <is>
+          <t>待补充</t>
         </is>
       </c>
     </row>
@@ -1641,9 +1636,9 @@
           <t>2025-08-19</t>
         </is>
       </c>
-      <c r="D54" t="inlineStr">
-        <is>
-          <t>2234.59万</t>
+      <c r="D54" s="2" t="inlineStr">
+        <is>
+          <t>待补充</t>
         </is>
       </c>
     </row>
@@ -1663,9 +1658,9 @@
           <t>获取失败</t>
         </is>
       </c>
-      <c r="D55" s="3" t="inlineStr">
-        <is>
-          <t>获取失败</t>
+      <c r="D55" s="2" t="inlineStr">
+        <is>
+          <t>待补充</t>
         </is>
       </c>
     </row>
@@ -1685,9 +1680,9 @@
           <t>2025-10-23</t>
         </is>
       </c>
-      <c r="D56" t="inlineStr">
-        <is>
-          <t>2647.94万</t>
+      <c r="D56" s="2" t="inlineStr">
+        <is>
+          <t>待补充</t>
         </is>
       </c>
     </row>
@@ -1707,9 +1702,9 @@
           <t>2025-07-29</t>
         </is>
       </c>
-      <c r="D57" t="inlineStr">
-        <is>
-          <t>1959.58万</t>
+      <c r="D57" s="2" t="inlineStr">
+        <is>
+          <t>待补充</t>
         </is>
       </c>
     </row>
@@ -1729,9 +1724,9 @@
           <t>2025-09-02</t>
         </is>
       </c>
-      <c r="D58" t="inlineStr">
-        <is>
-          <t>3375.37万</t>
+      <c r="D58" s="2" t="inlineStr">
+        <is>
+          <t>待补充</t>
         </is>
       </c>
     </row>
@@ -1751,9 +1746,9 @@
           <t>2025-08-19</t>
         </is>
       </c>
-      <c r="D59" t="inlineStr">
-        <is>
-          <t>737.52万</t>
+      <c r="D59" s="2" t="inlineStr">
+        <is>
+          <t>待补充</t>
         </is>
       </c>
     </row>
@@ -1773,9 +1768,9 @@
           <t>2025-09-30</t>
         </is>
       </c>
-      <c r="D60" t="inlineStr">
-        <is>
-          <t>1.66亿</t>
+      <c r="D60" s="2" t="inlineStr">
+        <is>
+          <t>待补充</t>
         </is>
       </c>
     </row>
@@ -1795,9 +1790,9 @@
           <t>2025-12-30</t>
         </is>
       </c>
-      <c r="D61" t="inlineStr">
-        <is>
-          <t>9.34亿</t>
+      <c r="D61" s="2" t="inlineStr">
+        <is>
+          <t>待补充</t>
         </is>
       </c>
     </row>
@@ -1817,9 +1812,9 @@
           <t>2025-10-15</t>
         </is>
       </c>
-      <c r="D62" t="inlineStr">
-        <is>
-          <t>1372.07万</t>
+      <c r="D62" s="2" t="inlineStr">
+        <is>
+          <t>待补充</t>
         </is>
       </c>
     </row>
@@ -1839,9 +1834,9 @@
           <t>2025-10-28</t>
         </is>
       </c>
-      <c r="D63" t="inlineStr">
-        <is>
-          <t>1363.58万</t>
+      <c r="D63" s="2" t="inlineStr">
+        <is>
+          <t>待补充</t>
         </is>
       </c>
     </row>
@@ -1861,9 +1856,9 @@
           <t>2025-11-21</t>
         </is>
       </c>
-      <c r="D64" t="inlineStr">
-        <is>
-          <t>2.31亿</t>
+      <c r="D64" s="2" t="inlineStr">
+        <is>
+          <t>待补充</t>
         </is>
       </c>
     </row>
@@ -1883,9 +1878,9 @@
           <t>获取失败</t>
         </is>
       </c>
-      <c r="D65" s="3" t="inlineStr">
-        <is>
-          <t>获取失败</t>
+      <c r="D65" s="2" t="inlineStr">
+        <is>
+          <t>待补充</t>
         </is>
       </c>
     </row>
@@ -1905,9 +1900,9 @@
           <t>获取失败</t>
         </is>
       </c>
-      <c r="D66" s="3" t="inlineStr">
-        <is>
-          <t>获取失败</t>
+      <c r="D66" s="2" t="inlineStr">
+        <is>
+          <t>待补充</t>
         </is>
       </c>
     </row>
@@ -1927,9 +1922,9 @@
           <t>2009-12-16</t>
         </is>
       </c>
-      <c r="D67" t="inlineStr">
-        <is>
-          <t>46.17亿</t>
+      <c r="D67" s="2" t="inlineStr">
+        <is>
+          <t>待补充</t>
         </is>
       </c>
     </row>
@@ -1949,9 +1944,9 @@
           <t>2012-07-05</t>
         </is>
       </c>
-      <c r="D68" t="inlineStr">
-        <is>
-          <t>9.35亿</t>
+      <c r="D68" s="2" t="inlineStr">
+        <is>
+          <t>待补充</t>
         </is>
       </c>
     </row>
@@ -1971,9 +1966,9 @@
           <t>获取失败</t>
         </is>
       </c>
-      <c r="D69" s="3" t="inlineStr">
-        <is>
-          <t>获取失败</t>
+      <c r="D69" s="2" t="inlineStr">
+        <is>
+          <t>待补充</t>
         </is>
       </c>
     </row>
@@ -1993,9 +1988,9 @@
           <t>2010-04-23</t>
         </is>
       </c>
-      <c r="D70" t="inlineStr">
-        <is>
-          <t>5.39亿</t>
+      <c r="D70" s="2" t="inlineStr">
+        <is>
+          <t>待补充</t>
         </is>
       </c>
     </row>
@@ -2015,9 +2010,9 @@
           <t>2010-11-02</t>
         </is>
       </c>
-      <c r="D71" t="inlineStr">
-        <is>
-          <t>39.43亿</t>
+      <c r="D71" s="2" t="inlineStr">
+        <is>
+          <t>待补充</t>
         </is>
       </c>
     </row>
@@ -2037,9 +2032,9 @@
           <t>2011-05-06</t>
         </is>
       </c>
-      <c r="D72" t="inlineStr">
-        <is>
-          <t>2.89亿</t>
+      <c r="D72" s="2" t="inlineStr">
+        <is>
+          <t>待补充</t>
         </is>
       </c>
     </row>
@@ -2059,9 +2054,9 @@
           <t>2012-05-07</t>
         </is>
       </c>
-      <c r="D73" t="inlineStr">
-        <is>
-          <t>1.54亿</t>
+      <c r="D73" s="2" t="inlineStr">
+        <is>
+          <t>待补充</t>
         </is>
       </c>
     </row>
@@ -2081,9 +2076,9 @@
           <t>2013-07-26</t>
         </is>
       </c>
-      <c r="D74" t="inlineStr">
-        <is>
-          <t>9469.08万</t>
+      <c r="D74" s="2" t="inlineStr">
+        <is>
+          <t>待补充</t>
         </is>
       </c>
     </row>
@@ -2103,9 +2098,9 @@
           <t>2004-05-21</t>
         </is>
       </c>
-      <c r="D75" t="inlineStr">
-        <is>
-          <t>7.98亿</t>
+      <c r="D75" s="2" t="inlineStr">
+        <is>
+          <t>待补充</t>
         </is>
       </c>
     </row>
@@ -2125,9 +2120,9 @@
           <t>2004-11-29</t>
         </is>
       </c>
-      <c r="D76" t="inlineStr">
-        <is>
-          <t>8.07亿</t>
+      <c r="D76" s="2" t="inlineStr">
+        <is>
+          <t>待补充</t>
         </is>
       </c>
     </row>
@@ -2147,9 +2142,9 @@
           <t>2011-04-07</t>
         </is>
       </c>
-      <c r="D77" t="inlineStr">
-        <is>
-          <t>3.53亿</t>
+      <c r="D77" s="2" t="inlineStr">
+        <is>
+          <t>待补充</t>
         </is>
       </c>
     </row>
@@ -2169,9 +2164,9 @@
           <t>2009-09-03</t>
         </is>
       </c>
-      <c r="D78" t="inlineStr">
-        <is>
-          <t>2.32亿</t>
+      <c r="D78" s="2" t="inlineStr">
+        <is>
+          <t>待补充</t>
         </is>
       </c>
     </row>
@@ -2191,9 +2186,9 @@
           <t>2010-12-10</t>
         </is>
       </c>
-      <c r="D79" t="inlineStr">
-        <is>
-          <t>2.36亿</t>
+      <c r="D79" s="2" t="inlineStr">
+        <is>
+          <t>待补充</t>
         </is>
       </c>
     </row>
@@ -2213,9 +2208,9 @@
           <t>获取失败</t>
         </is>
       </c>
-      <c r="D80" s="3" t="inlineStr">
-        <is>
-          <t>获取失败</t>
+      <c r="D80" s="2" t="inlineStr">
+        <is>
+          <t>待补充</t>
         </is>
       </c>
     </row>
@@ -2235,9 +2230,9 @@
           <t>获取失败</t>
         </is>
       </c>
-      <c r="D81" s="3" t="inlineStr">
-        <is>
-          <t>获取失败</t>
+      <c r="D81" s="2" t="inlineStr">
+        <is>
+          <t>待补充</t>
         </is>
       </c>
     </row>
@@ -2257,9 +2252,9 @@
           <t>获取失败</t>
         </is>
       </c>
-      <c r="D82" s="3" t="inlineStr">
-        <is>
-          <t>获取失败</t>
+      <c r="D82" s="2" t="inlineStr">
+        <is>
+          <t>待补充</t>
         </is>
       </c>
     </row>
@@ -2279,9 +2274,9 @@
           <t>获取失败</t>
         </is>
       </c>
-      <c r="D83" s="3" t="inlineStr">
-        <is>
-          <t>获取失败</t>
+      <c r="D83" s="2" t="inlineStr">
+        <is>
+          <t>待补充</t>
         </is>
       </c>
     </row>
@@ -2301,9 +2296,9 @@
           <t>2017-03-21</t>
         </is>
       </c>
-      <c r="D84" t="inlineStr">
-        <is>
-          <t>2.14亿</t>
+      <c r="D84" s="2" t="inlineStr">
+        <is>
+          <t>待补充</t>
         </is>
       </c>
     </row>
@@ -2323,6 +2318,7 @@
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
     <col width="40" customWidth="1" min="2" max="2"/>
+    <col width="11.1328125" bestFit="1" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2363,9 +2359,9 @@
           <t>2014-01-27</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>33.32亿</t>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>待补充</t>
         </is>
       </c>
     </row>
@@ -2385,9 +2381,9 @@
           <t>2015-02-16</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>13.03亿</t>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>待补充</t>
         </is>
       </c>
     </row>
@@ -2407,9 +2403,9 @@
           <t>2015-06-09</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>2758.73万</t>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>待补充</t>
         </is>
       </c>
     </row>
@@ -2429,9 +2425,9 @@
           <t>2015-06-30</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>19.13亿</t>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>待补充</t>
         </is>
       </c>
     </row>
@@ -2451,9 +2447,9 @@
           <t>2016-05-11</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>1.32亿</t>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>待补充</t>
         </is>
       </c>
     </row>
@@ -2473,9 +2469,9 @@
           <t>2015-12-31</t>
         </is>
       </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>1.80亿</t>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>待补充</t>
         </is>
       </c>
     </row>
@@ -2495,9 +2491,9 @@
           <t>2016-04-21</t>
         </is>
       </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>1.33亿</t>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>待补充</t>
         </is>
       </c>
     </row>
@@ -2517,9 +2513,9 @@
           <t>2016-11-23</t>
         </is>
       </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>4.08亿</t>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>待补充</t>
         </is>
       </c>
     </row>
@@ -2539,9 +2535,9 @@
           <t>2016-07-22</t>
         </is>
       </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>8.87亿</t>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>待补充</t>
         </is>
       </c>
     </row>
@@ -2561,9 +2557,9 @@
           <t>2017-08-01</t>
         </is>
       </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>8243.26万</t>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>待补充</t>
         </is>
       </c>
     </row>
@@ -2583,9 +2579,9 @@
           <t>2017-01-10</t>
         </is>
       </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>14.92亿</t>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>待补充</t>
         </is>
       </c>
     </row>
@@ -2605,9 +2601,9 @@
           <t>2017-05-17</t>
         </is>
       </c>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t>6.24亿</t>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>待补充</t>
         </is>
       </c>
     </row>
@@ -2627,9 +2623,9 @@
           <t>2017-08-30</t>
         </is>
       </c>
-      <c r="D14" t="inlineStr">
-        <is>
-          <t>2.44亿</t>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>待补充</t>
         </is>
       </c>
     </row>
@@ -2649,9 +2645,9 @@
           <t>2017-09-26</t>
         </is>
       </c>
-      <c r="D15" t="inlineStr">
-        <is>
-          <t>2.47亿</t>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>待补充</t>
         </is>
       </c>
     </row>
@@ -2671,9 +2667,9 @@
           <t>2018-04-19</t>
         </is>
       </c>
-      <c r="D16" t="inlineStr">
-        <is>
-          <t>3092.56万</t>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>待补充</t>
         </is>
       </c>
     </row>
@@ -2693,9 +2689,9 @@
           <t>2018-11-29</t>
         </is>
       </c>
-      <c r="D17" t="inlineStr">
-        <is>
-          <t>1156.65万</t>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>待补充</t>
         </is>
       </c>
     </row>
@@ -2715,9 +2711,9 @@
           <t>2018-08-01</t>
         </is>
       </c>
-      <c r="D18" t="inlineStr">
-        <is>
-          <t>9.74亿</t>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>待补充</t>
         </is>
       </c>
     </row>
@@ -2737,9 +2733,9 @@
           <t>2018-08-13</t>
         </is>
       </c>
-      <c r="D19" t="inlineStr">
-        <is>
-          <t>8.38亿</t>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t>待补充</t>
         </is>
       </c>
     </row>
@@ -2759,9 +2755,9 @@
           <t>2020-05-09</t>
         </is>
       </c>
-      <c r="D20" t="inlineStr">
-        <is>
-          <t>9843.42万</t>
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t>待补充</t>
         </is>
       </c>
     </row>
@@ -2781,9 +2777,9 @@
           <t>2019-01-03</t>
         </is>
       </c>
-      <c r="D21" t="inlineStr">
-        <is>
-          <t>14.95亿</t>
+      <c r="D21" s="2" t="inlineStr">
+        <is>
+          <t>待补充</t>
         </is>
       </c>
     </row>
@@ -2803,9 +2799,9 @@
           <t>2019-03-25</t>
         </is>
       </c>
-      <c r="D22" t="inlineStr">
-        <is>
-          <t>4.18亿</t>
+      <c r="D22" s="2" t="inlineStr">
+        <is>
+          <t>待补充</t>
         </is>
       </c>
     </row>
@@ -2825,9 +2821,9 @@
           <t>2019-05-23</t>
         </is>
       </c>
-      <c r="D23" t="inlineStr">
-        <is>
-          <t>6.47亿</t>
+      <c r="D23" s="2" t="inlineStr">
+        <is>
+          <t>待补充</t>
         </is>
       </c>
     </row>
@@ -2847,9 +2843,9 @@
           <t>2019-11-19</t>
         </is>
       </c>
-      <c r="D24" t="inlineStr">
-        <is>
-          <t>7830.15万</t>
+      <c r="D24" s="2" t="inlineStr">
+        <is>
+          <t>待补充</t>
         </is>
       </c>
     </row>
@@ -2869,9 +2865,9 @@
           <t>2020-03-25</t>
         </is>
       </c>
-      <c r="D25" t="inlineStr">
-        <is>
-          <t>38.06亿</t>
+      <c r="D25" s="2" t="inlineStr">
+        <is>
+          <t>待补充</t>
         </is>
       </c>
     </row>
@@ -2891,9 +2887,9 @@
           <t>2020-01-20</t>
         </is>
       </c>
-      <c r="D26" t="inlineStr">
-        <is>
-          <t>7786.00万</t>
+      <c r="D26" s="2" t="inlineStr">
+        <is>
+          <t>待补充</t>
         </is>
       </c>
     </row>
@@ -2913,9 +2909,9 @@
           <t>2020-05-27</t>
         </is>
       </c>
-      <c r="D27" t="inlineStr">
-        <is>
-          <t>1390.64万</t>
+      <c r="D27" s="2" t="inlineStr">
+        <is>
+          <t>待补充</t>
         </is>
       </c>
     </row>
@@ -2935,9 +2931,9 @@
           <t>2020-10-15</t>
         </is>
       </c>
-      <c r="D28" t="inlineStr">
-        <is>
-          <t>1.85亿</t>
+      <c r="D28" s="2" t="inlineStr">
+        <is>
+          <t>待补充</t>
         </is>
       </c>
     </row>
@@ -2957,9 +2953,9 @@
           <t>2020-07-01</t>
         </is>
       </c>
-      <c r="D29" t="inlineStr">
-        <is>
-          <t>3629.30万</t>
+      <c r="D29" s="2" t="inlineStr">
+        <is>
+          <t>待补充</t>
         </is>
       </c>
     </row>
@@ -2979,9 +2975,9 @@
           <t>2020-12-23</t>
         </is>
       </c>
-      <c r="D30" t="inlineStr">
-        <is>
-          <t>4.78亿</t>
+      <c r="D30" s="2" t="inlineStr">
+        <is>
+          <t>待补充</t>
         </is>
       </c>
     </row>
@@ -3001,9 +2997,9 @@
           <t>2020-09-27</t>
         </is>
       </c>
-      <c r="D31" t="inlineStr">
-        <is>
-          <t>1897.09万</t>
+      <c r="D31" s="2" t="inlineStr">
+        <is>
+          <t>待补充</t>
         </is>
       </c>
     </row>
@@ -3023,9 +3019,9 @@
           <t>获取失败</t>
         </is>
       </c>
-      <c r="D32" s="3" t="inlineStr">
-        <is>
-          <t>获取失败</t>
+      <c r="D32" s="2" t="inlineStr">
+        <is>
+          <t>待补充</t>
         </is>
       </c>
     </row>
@@ -3045,9 +3041,9 @@
           <t>2021-03-01</t>
         </is>
       </c>
-      <c r="D33" t="inlineStr">
-        <is>
-          <t>2701.93万</t>
+      <c r="D33" s="2" t="inlineStr">
+        <is>
+          <t>待补充</t>
         </is>
       </c>
     </row>
@@ -3067,9 +3063,9 @@
           <t>2021-06-15</t>
         </is>
       </c>
-      <c r="D34" t="inlineStr">
-        <is>
-          <t>4.72亿</t>
+      <c r="D34" s="2" t="inlineStr">
+        <is>
+          <t>待补充</t>
         </is>
       </c>
     </row>
@@ -3089,9 +3085,9 @@
           <t>2021-09-16</t>
         </is>
       </c>
-      <c r="D35" t="inlineStr">
-        <is>
-          <t>4901.87万</t>
+      <c r="D35" s="2" t="inlineStr">
+        <is>
+          <t>待补充</t>
         </is>
       </c>
     </row>
@@ -3111,9 +3107,9 @@
           <t>2021-08-10</t>
         </is>
       </c>
-      <c r="D36" t="inlineStr">
-        <is>
-          <t>3505.66万</t>
+      <c r="D36" s="2" t="inlineStr">
+        <is>
+          <t>待补充</t>
         </is>
       </c>
     </row>
@@ -3133,9 +3129,9 @@
           <t>2021-08-11</t>
         </is>
       </c>
-      <c r="D37" t="inlineStr">
-        <is>
-          <t>9.12亿</t>
+      <c r="D37" s="2" t="inlineStr">
+        <is>
+          <t>待补充</t>
         </is>
       </c>
     </row>
@@ -3155,9 +3151,9 @@
           <t>2021-09-29</t>
         </is>
       </c>
-      <c r="D38" t="inlineStr">
-        <is>
-          <t>1.04亿</t>
+      <c r="D38" s="2" t="inlineStr">
+        <is>
+          <t>待补充</t>
         </is>
       </c>
     </row>
@@ -3177,9 +3173,9 @@
           <t>2021-12-01</t>
         </is>
       </c>
-      <c r="D39" t="inlineStr">
-        <is>
-          <t>9277.21万</t>
+      <c r="D39" s="2" t="inlineStr">
+        <is>
+          <t>待补充</t>
         </is>
       </c>
     </row>
@@ -3199,9 +3195,9 @@
           <t>2021-12-14</t>
         </is>
       </c>
-      <c r="D40" t="inlineStr">
-        <is>
-          <t>8935.54万</t>
+      <c r="D40" s="2" t="inlineStr">
+        <is>
+          <t>待补充</t>
         </is>
       </c>
     </row>
@@ -3221,9 +3217,9 @@
           <t>2021-12-15</t>
         </is>
       </c>
-      <c r="D41" t="inlineStr">
-        <is>
-          <t>24.84亿</t>
+      <c r="D41" s="2" t="inlineStr">
+        <is>
+          <t>待补充</t>
         </is>
       </c>
     </row>
@@ -3243,9 +3239,9 @@
           <t>2022-04-27</t>
         </is>
       </c>
-      <c r="D42" t="inlineStr">
-        <is>
-          <t>3.20亿</t>
+      <c r="D42" s="2" t="inlineStr">
+        <is>
+          <t>待补充</t>
         </is>
       </c>
     </row>
@@ -3265,9 +3261,9 @@
           <t>2022-01-11</t>
         </is>
       </c>
-      <c r="D43" t="inlineStr">
-        <is>
-          <t>10.23亿</t>
+      <c r="D43" s="2" t="inlineStr">
+        <is>
+          <t>待补充</t>
         </is>
       </c>
     </row>
@@ -3287,9 +3283,9 @@
           <t>2022-05-24</t>
         </is>
       </c>
-      <c r="D44" t="inlineStr">
-        <is>
-          <t>4339.94万</t>
+      <c r="D44" s="2" t="inlineStr">
+        <is>
+          <t>待补充</t>
         </is>
       </c>
     </row>
@@ -3309,9 +3305,9 @@
           <t>2022-05-06</t>
         </is>
       </c>
-      <c r="D45" t="inlineStr">
-        <is>
-          <t>18.60亿</t>
+      <c r="D45" s="2" t="inlineStr">
+        <is>
+          <t>待补充</t>
         </is>
       </c>
     </row>
@@ -3331,9 +3327,9 @@
           <t>2022-06-07</t>
         </is>
       </c>
-      <c r="D46" t="inlineStr">
-        <is>
-          <t>1.55亿</t>
+      <c r="D46" s="2" t="inlineStr">
+        <is>
+          <t>待补充</t>
         </is>
       </c>
     </row>
@@ -3353,9 +3349,9 @@
           <t>2022-12-23</t>
         </is>
       </c>
-      <c r="D47" t="inlineStr">
-        <is>
-          <t>1.09亿</t>
+      <c r="D47" s="2" t="inlineStr">
+        <is>
+          <t>待补充</t>
         </is>
       </c>
     </row>
@@ -3375,9 +3371,9 @@
           <t>2022-10-25</t>
         </is>
       </c>
-      <c r="D48" t="inlineStr">
-        <is>
-          <t>559.34万</t>
+      <c r="D48" s="2" t="inlineStr">
+        <is>
+          <t>待补充</t>
         </is>
       </c>
     </row>
@@ -3397,9 +3393,9 @@
           <t>2023-02-22</t>
         </is>
       </c>
-      <c r="D49" t="inlineStr">
-        <is>
-          <t>3486.24万</t>
+      <c r="D49" s="2" t="inlineStr">
+        <is>
+          <t>待补充</t>
         </is>
       </c>
     </row>
@@ -3419,9 +3415,9 @@
           <t>2023-08-17</t>
         </is>
       </c>
-      <c r="D50" t="inlineStr">
-        <is>
-          <t>2161.54万</t>
+      <c r="D50" s="2" t="inlineStr">
+        <is>
+          <t>待补充</t>
         </is>
       </c>
     </row>
@@ -3441,9 +3437,9 @@
           <t>2023-07-13</t>
         </is>
       </c>
-      <c r="D51" t="inlineStr">
-        <is>
-          <t>2935.08万</t>
+      <c r="D51" s="2" t="inlineStr">
+        <is>
+          <t>待补充</t>
         </is>
       </c>
     </row>
@@ -3463,9 +3459,9 @@
           <t>2023-12-26</t>
         </is>
       </c>
-      <c r="D52" t="inlineStr">
-        <is>
-          <t>2027.83万</t>
+      <c r="D52" s="2" t="inlineStr">
+        <is>
+          <t>待补充</t>
         </is>
       </c>
     </row>
@@ -3485,9 +3481,9 @@
           <t>2024-08-13</t>
         </is>
       </c>
-      <c r="D53" t="inlineStr">
-        <is>
-          <t>1.13亿</t>
+      <c r="D53" s="2" t="inlineStr">
+        <is>
+          <t>待补充</t>
         </is>
       </c>
     </row>
@@ -3507,9 +3503,9 @@
           <t>2024-07-19</t>
         </is>
       </c>
-      <c r="D54" t="inlineStr">
-        <is>
-          <t>1905.22万</t>
+      <c r="D54" s="2" t="inlineStr">
+        <is>
+          <t>待补充</t>
         </is>
       </c>
     </row>
@@ -3529,9 +3525,9 @@
           <t>2024-07-09</t>
         </is>
       </c>
-      <c r="D55" t="inlineStr">
-        <is>
-          <t>3421.12万</t>
+      <c r="D55" s="2" t="inlineStr">
+        <is>
+          <t>待补充</t>
         </is>
       </c>
     </row>
@@ -3551,9 +3547,9 @@
           <t>2024-06-21</t>
         </is>
       </c>
-      <c r="D56" t="inlineStr">
-        <is>
-          <t>7240.92万</t>
+      <c r="D56" s="2" t="inlineStr">
+        <is>
+          <t>待补充</t>
         </is>
       </c>
     </row>
@@ -3573,9 +3569,9 @@
           <t>2025-03-18</t>
         </is>
       </c>
-      <c r="D57" t="inlineStr">
-        <is>
-          <t>2143.25万</t>
+      <c r="D57" s="2" t="inlineStr">
+        <is>
+          <t>待补充</t>
         </is>
       </c>
     </row>
@@ -3595,9 +3591,9 @@
           <t>获取失败</t>
         </is>
       </c>
-      <c r="D58" s="3" t="inlineStr">
-        <is>
-          <t>获取失败</t>
+      <c r="D58" s="2" t="inlineStr">
+        <is>
+          <t>待补充</t>
         </is>
       </c>
     </row>
@@ -3617,9 +3613,9 @@
           <t>2025-10-31</t>
         </is>
       </c>
-      <c r="D59" t="inlineStr">
-        <is>
-          <t>1.10亿</t>
+      <c r="D59" s="2" t="inlineStr">
+        <is>
+          <t>待补充</t>
         </is>
       </c>
     </row>
@@ -3639,9 +3635,9 @@
           <t>获取失败</t>
         </is>
       </c>
-      <c r="D60" s="3" t="inlineStr">
-        <is>
-          <t>获取失败</t>
+      <c r="D60" s="2" t="inlineStr">
+        <is>
+          <t>待补充</t>
         </is>
       </c>
     </row>
@@ -3661,9 +3657,9 @@
           <t>2025-07-23</t>
         </is>
       </c>
-      <c r="D61" t="inlineStr">
-        <is>
-          <t>6399.46万</t>
+      <c r="D61" s="2" t="inlineStr">
+        <is>
+          <t>待补充</t>
         </is>
       </c>
     </row>
@@ -3683,9 +3679,9 @@
           <t>2025-04-17</t>
         </is>
       </c>
-      <c r="D62" t="inlineStr">
-        <is>
-          <t>7658.44万</t>
+      <c r="D62" s="2" t="inlineStr">
+        <is>
+          <t>待补充</t>
         </is>
       </c>
     </row>
@@ -3705,9 +3701,9 @@
           <t>获取失败</t>
         </is>
       </c>
-      <c r="D63" s="3" t="inlineStr">
-        <is>
-          <t>获取失败</t>
+      <c r="D63" s="2" t="inlineStr">
+        <is>
+          <t>待补充</t>
         </is>
       </c>
     </row>
@@ -3727,9 +3723,9 @@
           <t>2025-09-12</t>
         </is>
       </c>
-      <c r="D64" t="inlineStr">
-        <is>
-          <t>3856.85万</t>
+      <c r="D64" s="2" t="inlineStr">
+        <is>
+          <t>待补充</t>
         </is>
       </c>
     </row>
@@ -3749,9 +3745,9 @@
           <t>2025-12-16</t>
         </is>
       </c>
-      <c r="D65" t="inlineStr">
-        <is>
-          <t>4.35亿</t>
+      <c r="D65" s="2" t="inlineStr">
+        <is>
+          <t>待补充</t>
         </is>
       </c>
     </row>
@@ -3771,9 +3767,9 @@
           <t>获取失败</t>
         </is>
       </c>
-      <c r="D66" s="3" t="inlineStr">
-        <is>
-          <t>获取失败</t>
+      <c r="D66" s="2" t="inlineStr">
+        <is>
+          <t>待补充</t>
         </is>
       </c>
     </row>
@@ -3793,9 +3789,9 @@
           <t>2025-11-25</t>
         </is>
       </c>
-      <c r="D67" t="inlineStr">
-        <is>
-          <t>3404.98万</t>
+      <c r="D67" s="2" t="inlineStr">
+        <is>
+          <t>待补充</t>
         </is>
       </c>
     </row>
@@ -3815,9 +3811,9 @@
           <t>获取失败</t>
         </is>
       </c>
-      <c r="D68" s="3" t="inlineStr">
-        <is>
-          <t>获取失败</t>
+      <c r="D68" s="2" t="inlineStr">
+        <is>
+          <t>待补充</t>
         </is>
       </c>
     </row>
@@ -3837,9 +3833,9 @@
           <t>2025-12-19</t>
         </is>
       </c>
-      <c r="D69" t="inlineStr">
-        <is>
-          <t>8088.65万</t>
+      <c r="D69" s="2" t="inlineStr">
+        <is>
+          <t>待补充</t>
         </is>
       </c>
     </row>
@@ -3859,9 +3855,9 @@
           <t>2026-02-10</t>
         </is>
       </c>
-      <c r="D70" t="inlineStr">
-        <is>
-          <t>5.78亿</t>
+      <c r="D70" s="2" t="inlineStr">
+        <is>
+          <t>待补充</t>
         </is>
       </c>
     </row>
@@ -3881,9 +3877,9 @@
           <t>获取失败</t>
         </is>
       </c>
-      <c r="D71" s="3" t="inlineStr">
-        <is>
-          <t>获取失败</t>
+      <c r="D71" s="2" t="inlineStr">
+        <is>
+          <t>待补充</t>
         </is>
       </c>
     </row>
@@ -3903,9 +3899,9 @@
           <t>获取失败</t>
         </is>
       </c>
-      <c r="D72" s="3" t="inlineStr">
-        <is>
-          <t>获取失败</t>
+      <c r="D72" s="2" t="inlineStr">
+        <is>
+          <t>待补充</t>
         </is>
       </c>
     </row>
@@ -3925,9 +3921,9 @@
           <t>获取失败</t>
         </is>
       </c>
-      <c r="D73" s="3" t="inlineStr">
-        <is>
-          <t>获取失败</t>
+      <c r="D73" s="2" t="inlineStr">
+        <is>
+          <t>待补充</t>
         </is>
       </c>
     </row>
@@ -3947,9 +3943,9 @@
           <t>2011-10-12</t>
         </is>
       </c>
-      <c r="D74" t="inlineStr">
-        <is>
-          <t>39.47亿</t>
+      <c r="D74" s="2" t="inlineStr">
+        <is>
+          <t>待补充</t>
         </is>
       </c>
     </row>
@@ -3969,9 +3965,9 @@
           <t>2011-12-01</t>
         </is>
       </c>
-      <c r="D75" t="inlineStr">
-        <is>
-          <t>1.75亿</t>
+      <c r="D75" s="2" t="inlineStr">
+        <is>
+          <t>待补充</t>
         </is>
       </c>
     </row>
@@ -3991,9 +3987,9 @@
           <t>2015-04-15</t>
         </is>
       </c>
-      <c r="D76" t="inlineStr">
-        <is>
-          <t>10.72亿</t>
+      <c r="D76" s="2" t="inlineStr">
+        <is>
+          <t>待补充</t>
         </is>
       </c>
     </row>
@@ -4013,9 +4009,9 @@
           <t>2012-05-25</t>
         </is>
       </c>
-      <c r="D77" t="inlineStr">
-        <is>
-          <t>2978.59万</t>
+      <c r="D77" s="2" t="inlineStr">
+        <is>
+          <t>待补充</t>
         </is>
       </c>
     </row>
@@ -4035,9 +4031,9 @@
           <t>获取失败</t>
         </is>
       </c>
-      <c r="D78" s="3" t="inlineStr">
-        <is>
-          <t>获取失败</t>
+      <c r="D78" s="2" t="inlineStr">
+        <is>
+          <t>待补充</t>
         </is>
       </c>
     </row>
@@ -4057,9 +4053,9 @@
           <t>获取失败</t>
         </is>
       </c>
-      <c r="D79" s="3" t="inlineStr">
-        <is>
-          <t>获取失败</t>
+      <c r="D79" s="2" t="inlineStr">
+        <is>
+          <t>待补充</t>
         </is>
       </c>
     </row>
@@ -4079,9 +4075,9 @@
           <t>获取失败</t>
         </is>
       </c>
-      <c r="D80" s="3" t="inlineStr">
-        <is>
-          <t>获取失败</t>
+      <c r="D80" s="2" t="inlineStr">
+        <is>
+          <t>待补充</t>
         </is>
       </c>
     </row>
@@ -4101,9 +4097,9 @@
           <t>获取失败</t>
         </is>
       </c>
-      <c r="D81" s="3" t="inlineStr">
-        <is>
-          <t>获取失败</t>
+      <c r="D81" s="2" t="inlineStr">
+        <is>
+          <t>待补充</t>
         </is>
       </c>
     </row>
@@ -4123,9 +4119,9 @@
           <t>获取失败</t>
         </is>
       </c>
-      <c r="D82" s="3" t="inlineStr">
-        <is>
-          <t>获取失败</t>
+      <c r="D82" s="2" t="inlineStr">
+        <is>
+          <t>待补充</t>
         </is>
       </c>
     </row>
@@ -4145,9 +4141,9 @@
           <t>2011-11-22</t>
         </is>
       </c>
-      <c r="D83" t="inlineStr">
-        <is>
-          <t>5731.22万</t>
+      <c r="D83" s="2" t="inlineStr">
+        <is>
+          <t>待补充</t>
         </is>
       </c>
     </row>
@@ -4167,6 +4163,7 @@
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
     <col width="40" customWidth="1" min="2" max="2"/>
+    <col width="11.1328125" bestFit="1" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -4207,9 +4204,9 @@
           <t>2016-12-22</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>3575.34万</t>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>待补充</t>
         </is>
       </c>
     </row>
@@ -4229,9 +4226,9 @@
           <t>2017-03-03</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>10.48亿</t>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>待补充</t>
         </is>
       </c>
     </row>
@@ -4251,9 +4248,9 @@
           <t>2018-01-30</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>8.49亿</t>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>待补充</t>
         </is>
       </c>
     </row>
@@ -4273,9 +4270,9 @@
           <t>2018-11-22</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>6.11亿</t>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>待补充</t>
         </is>
       </c>
     </row>
@@ -4295,9 +4292,9 @@
           <t>2021-12-07</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>1.00亿</t>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>待补充</t>
         </is>
       </c>
     </row>
@@ -4317,9 +4314,9 @@
           <t>2022-01-04</t>
         </is>
       </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>8.57亿</t>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>待补充</t>
         </is>
       </c>
     </row>
@@ -4339,9 +4336,9 @@
           <t>2022-01-26</t>
         </is>
       </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>7012.16万</t>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>待补充</t>
         </is>
       </c>
     </row>
@@ -4361,9 +4358,9 @@
           <t>2022-07-12</t>
         </is>
       </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>2867.73万</t>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>待补充</t>
         </is>
       </c>
     </row>
@@ -4383,9 +4380,9 @@
           <t>2022-04-29</t>
         </is>
       </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>3.02亿</t>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>待补充</t>
         </is>
       </c>
     </row>
@@ -4405,9 +4402,9 @@
           <t>2022-04-27</t>
         </is>
       </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>4686.89万</t>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>待补充</t>
         </is>
       </c>
     </row>
@@ -4427,9 +4424,9 @@
           <t>2022-06-28</t>
         </is>
       </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>2.06亿</t>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>待补充</t>
         </is>
       </c>
     </row>
@@ -4449,9 +4446,9 @@
           <t>2022-08-16</t>
         </is>
       </c>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t>11.75亿</t>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>待补充</t>
         </is>
       </c>
     </row>
@@ -4471,9 +4468,9 @@
           <t>2022-12-06</t>
         </is>
       </c>
-      <c r="D14" t="inlineStr">
-        <is>
-          <t>5529.41万</t>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>待补充</t>
         </is>
       </c>
     </row>
@@ -4493,9 +4490,9 @@
           <t>2022-12-26</t>
         </is>
       </c>
-      <c r="D15" t="inlineStr">
-        <is>
-          <t>20.08亿</t>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>待补充</t>
         </is>
       </c>
     </row>
@@ -4515,9 +4512,9 @@
           <t>2023-04-13</t>
         </is>
       </c>
-      <c r="D16" t="inlineStr">
-        <is>
-          <t>3.94亿</t>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>待补充</t>
         </is>
       </c>
     </row>
@@ -4537,9 +4534,9 @@
           <t>2023-03-28</t>
         </is>
       </c>
-      <c r="D17" t="inlineStr">
-        <is>
-          <t>8.48亿</t>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>待补充</t>
         </is>
       </c>
     </row>
@@ -4559,9 +4556,9 @@
           <t>2022-12-05</t>
         </is>
       </c>
-      <c r="D18" t="inlineStr">
-        <is>
-          <t>1.49亿</t>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>待补充</t>
         </is>
       </c>
     </row>
@@ -4581,9 +4578,9 @@
           <t>2023-02-14</t>
         </is>
       </c>
-      <c r="D19" t="inlineStr">
-        <is>
-          <t>3756.60万</t>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t>待补充</t>
         </is>
       </c>
     </row>
@@ -4603,9 +4600,9 @@
           <t>2023-04-25</t>
         </is>
       </c>
-      <c r="D20" t="inlineStr">
-        <is>
-          <t>5.59亿</t>
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t>待补充</t>
         </is>
       </c>
     </row>
@@ -4625,9 +4622,9 @@
           <t>2022-11-28</t>
         </is>
       </c>
-      <c r="D21" t="inlineStr">
-        <is>
-          <t>1.14亿</t>
+      <c r="D21" s="2" t="inlineStr">
+        <is>
+          <t>待补充</t>
         </is>
       </c>
     </row>
@@ -4647,9 +4644,9 @@
           <t>2023-07-18</t>
         </is>
       </c>
-      <c r="D22" t="inlineStr">
-        <is>
-          <t>1350.89万</t>
+      <c r="D22" s="2" t="inlineStr">
+        <is>
+          <t>待补充</t>
         </is>
       </c>
     </row>
@@ -4669,9 +4666,9 @@
           <t>获取失败</t>
         </is>
       </c>
-      <c r="D23" s="3" t="inlineStr">
-        <is>
-          <t>获取失败</t>
+      <c r="D23" s="2" t="inlineStr">
+        <is>
+          <t>待补充</t>
         </is>
       </c>
     </row>
@@ -4691,9 +4688,9 @@
           <t>2023-08-25</t>
         </is>
       </c>
-      <c r="D24" t="inlineStr">
-        <is>
-          <t>2.88亿</t>
+      <c r="D24" s="2" t="inlineStr">
+        <is>
+          <t>待补充</t>
         </is>
       </c>
     </row>
@@ -4713,9 +4710,9 @@
           <t>2023-03-14</t>
         </is>
       </c>
-      <c r="D25" t="inlineStr">
-        <is>
-          <t>1.33亿</t>
+      <c r="D25" s="2" t="inlineStr">
+        <is>
+          <t>待补充</t>
         </is>
       </c>
     </row>
@@ -4735,9 +4732,9 @@
           <t>2023-03-22</t>
         </is>
       </c>
-      <c r="D26" t="inlineStr">
-        <is>
-          <t>2.01亿</t>
+      <c r="D26" s="2" t="inlineStr">
+        <is>
+          <t>待补充</t>
         </is>
       </c>
     </row>
@@ -4757,9 +4754,9 @@
           <t>2023-03-02</t>
         </is>
       </c>
-      <c r="D27" t="inlineStr">
-        <is>
-          <t>2.64亿</t>
+      <c r="D27" s="2" t="inlineStr">
+        <is>
+          <t>待补充</t>
         </is>
       </c>
     </row>
@@ -4779,9 +4776,9 @@
           <t>2023-05-19</t>
         </is>
       </c>
-      <c r="D28" t="inlineStr">
-        <is>
-          <t>14.72亿</t>
+      <c r="D28" s="2" t="inlineStr">
+        <is>
+          <t>待补充</t>
         </is>
       </c>
     </row>
@@ -4801,9 +4798,9 @@
           <t>2023-04-20</t>
         </is>
       </c>
-      <c r="D29" t="inlineStr">
-        <is>
-          <t>3.87亿</t>
+      <c r="D29" s="2" t="inlineStr">
+        <is>
+          <t>待补充</t>
         </is>
       </c>
     </row>
@@ -4823,9 +4820,9 @@
           <t>2023-06-08</t>
         </is>
       </c>
-      <c r="D30" t="inlineStr">
-        <is>
-          <t>1698.95万</t>
+      <c r="D30" s="2" t="inlineStr">
+        <is>
+          <t>待补充</t>
         </is>
       </c>
     </row>
@@ -4845,9 +4842,9 @@
           <t>2023-04-25</t>
         </is>
       </c>
-      <c r="D31" t="inlineStr">
-        <is>
-          <t>2.08亿</t>
+      <c r="D31" s="2" t="inlineStr">
+        <is>
+          <t>待补充</t>
         </is>
       </c>
     </row>
@@ -4867,9 +4864,9 @@
           <t>2023-09-26</t>
         </is>
       </c>
-      <c r="D32" t="inlineStr">
-        <is>
-          <t>1012.36万</t>
+      <c r="D32" s="2" t="inlineStr">
+        <is>
+          <t>待补充</t>
         </is>
       </c>
     </row>
@@ -4889,9 +4886,9 @@
           <t>2023-08-01</t>
         </is>
       </c>
-      <c r="D33" t="inlineStr">
-        <is>
-          <t>7929.09万</t>
+      <c r="D33" s="2" t="inlineStr">
+        <is>
+          <t>待补充</t>
         </is>
       </c>
     </row>
@@ -4911,9 +4908,9 @@
           <t>2023-10-26</t>
         </is>
       </c>
-      <c r="D34" t="inlineStr">
-        <is>
-          <t>1683.44万</t>
+      <c r="D34" s="2" t="inlineStr">
+        <is>
+          <t>待补充</t>
         </is>
       </c>
     </row>
@@ -4933,9 +4930,9 @@
           <t>2023-09-19</t>
         </is>
       </c>
-      <c r="D35" t="inlineStr">
-        <is>
-          <t>8.38亿</t>
+      <c r="D35" s="2" t="inlineStr">
+        <is>
+          <t>待补充</t>
         </is>
       </c>
     </row>
@@ -4955,9 +4952,9 @@
           <t>2023-11-07</t>
         </is>
       </c>
-      <c r="D36" t="inlineStr">
-        <is>
-          <t>453.93万</t>
+      <c r="D36" s="2" t="inlineStr">
+        <is>
+          <t>待补充</t>
         </is>
       </c>
     </row>
@@ -4977,9 +4974,9 @@
           <t>2024-04-29</t>
         </is>
       </c>
-      <c r="D37" t="inlineStr">
-        <is>
-          <t>1038.82万</t>
+      <c r="D37" s="2" t="inlineStr">
+        <is>
+          <t>待补充</t>
         </is>
       </c>
     </row>
@@ -4999,17 +4996,15 @@
           <t>2023-12-12</t>
         </is>
       </c>
-      <c r="D38" t="inlineStr">
-        <is>
-          <t>3.02亿</t>
+      <c r="D38" s="2" t="inlineStr">
+        <is>
+          <t>待补充</t>
         </is>
       </c>
     </row>
     <row r="39">
-      <c r="A39" t="inlineStr">
-        <is>
-          <t>159677</t>
-        </is>
+      <c r="A39" t="n">
+        <v>159677</v>
       </c>
       <c r="B39" t="inlineStr">
         <is>
@@ -5021,9 +5016,9 @@
           <t>获取失败</t>
         </is>
       </c>
-      <c r="D39" s="3" t="inlineStr">
-        <is>
-          <t>获取失败</t>
+      <c r="D39" s="2" t="inlineStr">
+        <is>
+          <t>待补充</t>
         </is>
       </c>
     </row>
@@ -5043,9 +5038,9 @@
           <t>获取失败</t>
         </is>
       </c>
-      <c r="D40" s="3" t="inlineStr">
-        <is>
-          <t>获取失败</t>
+      <c r="D40" s="2" t="inlineStr">
+        <is>
+          <t>待补充</t>
         </is>
       </c>
     </row>
@@ -5065,9 +5060,9 @@
           <t>获取失败</t>
         </is>
       </c>
-      <c r="D41" s="3" t="inlineStr">
-        <is>
-          <t>获取失败</t>
+      <c r="D41" s="2" t="inlineStr">
+        <is>
+          <t>待补充</t>
         </is>
       </c>
     </row>
@@ -5087,9 +5082,9 @@
           <t>获取失败</t>
         </is>
       </c>
-      <c r="D42" s="3" t="inlineStr">
-        <is>
-          <t>获取失败</t>
+      <c r="D42" s="2" t="inlineStr">
+        <is>
+          <t>待补充</t>
         </is>
       </c>
     </row>
@@ -5109,9 +5104,9 @@
           <t>2018-05-31</t>
         </is>
       </c>
-      <c r="D43" t="inlineStr">
-        <is>
-          <t>7.05亿</t>
+      <c r="D43" s="2" t="inlineStr">
+        <is>
+          <t>待补充</t>
         </is>
       </c>
     </row>
@@ -5131,9 +5126,9 @@
           <t>获取失败</t>
         </is>
       </c>
-      <c r="D44" s="3" t="inlineStr">
-        <is>
-          <t>获取失败</t>
+      <c r="D44" s="2" t="inlineStr">
+        <is>
+          <t>待补充</t>
         </is>
       </c>
     </row>
@@ -5153,9 +5148,9 @@
           <t>获取失败</t>
         </is>
       </c>
-      <c r="D45" s="3" t="inlineStr">
-        <is>
-          <t>获取失败</t>
+      <c r="D45" s="2" t="inlineStr">
+        <is>
+          <t>待补充</t>
         </is>
       </c>
     </row>
@@ -5175,9 +5170,9 @@
           <t>获取失败</t>
         </is>
       </c>
-      <c r="D46" s="3" t="inlineStr">
-        <is>
-          <t>获取失败</t>
+      <c r="D46" s="2" t="inlineStr">
+        <is>
+          <t>待补充</t>
         </is>
       </c>
     </row>
@@ -5197,9 +5192,9 @@
           <t>获取失败</t>
         </is>
       </c>
-      <c r="D47" s="3" t="inlineStr">
-        <is>
-          <t>获取失败</t>
+      <c r="D47" s="2" t="inlineStr">
+        <is>
+          <t>待补充</t>
         </is>
       </c>
     </row>
@@ -5219,6 +5214,7 @@
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
     <col width="40" customWidth="1" min="2" max="2"/>
+    <col width="11.1328125" bestFit="1" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -5259,9 +5255,9 @@
           <t>2025-03-20</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>670.64万</t>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>待补充</t>
         </is>
       </c>
     </row>
@@ -5281,9 +5277,9 @@
           <t>获取失败</t>
         </is>
       </c>
-      <c r="D3" s="3" t="inlineStr">
-        <is>
-          <t>获取失败</t>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>待补充</t>
         </is>
       </c>
     </row>
@@ -5303,9 +5299,9 @@
           <t>2025-09-16</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>6.98亿</t>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>待补充</t>
         </is>
       </c>
     </row>
@@ -5325,9 +5321,9 @@
           <t>获取失败</t>
         </is>
       </c>
-      <c r="D5" s="3" t="inlineStr">
-        <is>
-          <t>获取失败</t>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>待补充</t>
         </is>
       </c>
     </row>
@@ -5347,9 +5343,9 @@
           <t>2025-11-12</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>1.70亿</t>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>待补充</t>
         </is>
       </c>
     </row>
@@ -5369,9 +5365,9 @@
           <t>2025-12-29</t>
         </is>
       </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>1002.50万</t>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>待补充</t>
         </is>
       </c>
     </row>
@@ -5391,9 +5387,9 @@
           <t>2025-12-16</t>
         </is>
       </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>5178.20万</t>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>待补充</t>
         </is>
       </c>
     </row>
@@ -5413,9 +5409,9 @@
           <t>获取失败</t>
         </is>
       </c>
-      <c r="D9" s="3" t="inlineStr">
-        <is>
-          <t>获取失败</t>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>待补充</t>
         </is>
       </c>
     </row>
@@ -5435,9 +5431,9 @@
           <t>2026-02-03</t>
         </is>
       </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>2237.80万</t>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>待补充</t>
         </is>
       </c>
     </row>
@@ -5457,9 +5453,9 @@
           <t>2026-04-14</t>
         </is>
       </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>6147.03万</t>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>待补充</t>
         </is>
       </c>
     </row>
@@ -5479,9 +5475,9 @@
           <t>获取失败</t>
         </is>
       </c>
-      <c r="D12" s="3" t="inlineStr">
-        <is>
-          <t>获取失败</t>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>待补充</t>
         </is>
       </c>
     </row>
@@ -5501,9 +5497,9 @@
           <t>获取失败</t>
         </is>
       </c>
-      <c r="D13" s="3" t="inlineStr">
-        <is>
-          <t>获取失败</t>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>待补充</t>
         </is>
       </c>
     </row>
@@ -5523,9 +5519,9 @@
           <t>获取失败</t>
         </is>
       </c>
-      <c r="D14" s="3" t="inlineStr">
-        <is>
-          <t>获取失败</t>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>待补充</t>
         </is>
       </c>
     </row>
@@ -5545,9 +5541,9 @@
           <t>获取失败</t>
         </is>
       </c>
-      <c r="D15" s="3" t="inlineStr">
-        <is>
-          <t>获取失败</t>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>待补充</t>
         </is>
       </c>
     </row>
@@ -5567,9 +5563,9 @@
           <t>获取失败</t>
         </is>
       </c>
-      <c r="D16" s="3" t="inlineStr">
-        <is>
-          <t>获取失败</t>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>待补充</t>
         </is>
       </c>
     </row>
@@ -5589,9 +5585,9 @@
           <t>获取失败</t>
         </is>
       </c>
-      <c r="D17" s="3" t="inlineStr">
-        <is>
-          <t>获取失败</t>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>待补充</t>
         </is>
       </c>
     </row>

</xml_diff>